<commit_message>
HIDROCARBUROS: Ucayali 2025 en texto continuo, con el VAB del INEI 2015–2025
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DrqJkouEJ5iuRzFV6cVyPN
</commit_message>
<xml_diff>
--- a/HIDROCARBUROS/analisis/Ucayali_petroleo_2025_evidencia.xlsx
+++ b/HIDROCARBUROS/analisis/Ucayali_petroleo_2025_evidencia.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Regalias_2024_2025" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Canon_Ucayali" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Canon_por_lote_2025" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="INEI_participacion" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="VAB_INEI_2015_2025" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Contratos_Ucayali" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="138">
   <si>
     <t xml:space="preserve">Ucayali: producción fiscalizada de los lotes 31-C y 131, 2016–2025</t>
   </si>
@@ -318,15 +318,51 @@
     <t xml:space="preserve">El lote 131 figura en otra zona («Provincia Puerto Inca – Huánuco»): su canon va íntegro a Huánuco.</t>
   </si>
   <si>
-    <t xml:space="preserve">Participación de Ucayali en el VAB nacional (estructura %, INEI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente: INEI, «Producto Bruto Interno por Actividades Económicas, según Departamentos», valores a precios constantes de 2007, estructura porcentual: Cuadro N° 74 (2007) y Cuadro N° 180 (2025)</t>
+    <t xml:space="preserve">Ucayali: VAB total y de extracción de petróleo, gas y minerales, 2015–2025 (miles de soles de 2007)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente: INEI, «Ucayali: Valor Agregado Bruto por Años, según Actividades Económicas», Cuadro N° 1, valores a precios constantes de 2007 (2023P y 2024P preliminares, 2025E estimado); estructura 2025 y crecimiento promedio 2016–2025 del cuadro resumen del INEI</t>
   </si>
   <si>
     <t xml:space="preserve">Extracción de petróleo, gas y minerales</t>
   </si>
   <si>
+    <t xml:space="preserve">VAB Ucayali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Participación de la extracción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAB sin extracción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crec. promedio anual 2016–2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INEI publicado (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contribución de la extracción al crecimiento 2025 (p.p.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Var. INEI publicada 2025 (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Participación de Ucayali en el VAB nacional (estructura %)</t>
+  </si>
+  <si>
     <t xml:space="preserve">VAB total</t>
   </si>
   <si>
@@ -336,7 +372,10 @@
     <t xml:space="preserve">2025 (Cuadro N° 180)</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE: serie del VAB de Ucayali 2014–2025 (INEI, «Ucayali: Valor Agregado Bruto por Años, según Actividades Económicas», cuadros 1 y 2). Sin ella no se calculan el crecimiento, el peso en la economía regional ni la contribución.</t>
+    <t xml:space="preserve">En 2025 la extracción es la penúltima actividad de Ucayali (1,9 % del VAB), solo por encima de electricidad, gas y agua (0,7 %), según el cuadro resumen del INEI.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INEI, «Producto Bruto Interno por Actividades Económicas, según Departamentos», estructura porcentual, cuadros 74 y 180.</t>
   </si>
   <si>
     <t xml:space="preserve">Contratos de licencia en fase de explotación con área en Ucayali, al 31/12/2025</t>
@@ -2146,12 +2185,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2164,7 +2207,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>48</v>
       </c>
@@ -2172,34 +2215,444 @@
         <v>99</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>100</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B5" s="13" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>1</v>
+        <v>103</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>342484</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>4163474</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <f aca="false">B5/D5</f>
+        <v>0.0822591902819616</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <f aca="false">D5-B5</f>
+        <v>3820990</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B6" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>251895</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <f aca="false">B6/B5-1</f>
+        <v>-0.264505787131662</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>4176645</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <f aca="false">D6/D5-1</f>
+        <v>0.00316346397263434</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <f aca="false">B6/D6</f>
+        <v>0.0603103687289679</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <f aca="false">D6-B6</f>
+        <v>3924750</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <f aca="false">G6/G5-1</f>
+        <v>0.027155266043617</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>253330</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <f aca="false">B7/B6-1</f>
+        <v>0.00569681811866052</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>4305190</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <f aca="false">D7/D6-1</f>
+        <v>0.0307770950128632</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <f aca="false">B7/D7</f>
+        <v>0.058842931438566</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <f aca="false">D7-B7</f>
+        <v>4051860</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <f aca="false">G7/G6-1</f>
+        <v>0.0323867762277852</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>261501</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <f aca="false">B8/B7-1</f>
+        <v>0.0322543717680497</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>4440780</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <f aca="false">D8/D7-1</f>
+        <v>0.0314945449562041</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <f aca="false">B8/D8</f>
+        <v>0.0588862767351681</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <f aca="false">D8-B8</f>
+        <v>4179279</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <f aca="false">G8/G7-1</f>
+        <v>0.0314470391375812</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>259748</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <f aca="false">B9/B8-1</f>
+        <v>-0.00670360725197994</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>4625127</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <f aca="false">D9/D8-1</f>
+        <v>0.0415123018929107</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <f aca="false">B9/D9</f>
+        <v>0.0561601876013351</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <f aca="false">D9-B9</f>
+        <v>4365379</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <f aca="false">G9/G8-1</f>
+        <v>0.0445292118568776</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>168003</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <f aca="false">B10/B9-1</f>
+        <v>-0.353207724409813</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>4022097</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <f aca="false">D10/D9-1</f>
+        <v>-0.130381284665264</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <f aca="false">B10/D10</f>
+        <v>0.0417700020660864</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <f aca="false">D10-B10</f>
+        <v>3854094</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <f aca="false">G10/G9-1</f>
+        <v>-0.117122705726124</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>149669</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <f aca="false">B11/B10-1</f>
+        <v>-0.109129003648744</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>4571302</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <f aca="false">D11/D10-1</f>
+        <v>0.136546930618531</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <f aca="false">B11/D11</f>
+        <v>0.0327410002664449</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <f aca="false">D11-B11</f>
+        <v>4421633</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <f aca="false">G11/G10-1</f>
+        <v>0.147256138537358</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>143459</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <f aca="false">B12/B11-1</f>
+        <v>-0.0414915580380707</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>4730624</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <f aca="false">D12/D11-1</f>
+        <v>0.0348526524828157</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <f aca="false">B12/D12</f>
+        <v>0.0303255976378592</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <f aca="false">D12-B12</f>
+        <v>4587165</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <f aca="false">G12/G11-1</f>
+        <v>0.0374368474271836</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>132651</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <f aca="false">B13/B12-1</f>
+        <v>-0.0753385984845845</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>4789007</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <f aca="false">D13/D12-1</f>
+        <v>0.0123415008252612</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <f aca="false">B13/D13</f>
+        <v>0.0276990616217517</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <f aca="false">D13-B13</f>
+        <v>4656356</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <f aca="false">G13/G12-1</f>
+        <v>0.0150836082852917</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>113755</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <f aca="false">B14/B13-1</f>
+        <v>-0.142448982668808</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>4774634</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <f aca="false">D14/D13-1</f>
+        <v>-0.00300124848428918</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <f aca="false">B14/D14</f>
+        <v>0.0238248628062381</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <f aca="false">D14-B14</f>
+        <v>4660879</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <f aca="false">G14/G13-1</f>
+        <v>0.000971360437217461</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>93005</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <f aca="false">B15/B14-1</f>
+        <v>-0.182409564414751</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>4893850</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <f aca="false">D15/D14-1</f>
+        <v>0.0249686153954418</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <f aca="false">B15/D15</f>
+        <v>0.0190044647874373</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <f aca="false">D15-B15</f>
+        <v>4800845</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <f aca="false">G15/G14-1</f>
+        <v>0.0300299578684622</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="10" t="n">
+        <f aca="false">(B15/B5)^(1/10)-1</f>
+        <v>-0.122218141204513</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <f aca="false">(D15/D5)^(1/10)-1</f>
+        <v>0.016294276339671</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>-12.22</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>1.63</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="12" t="n">
+        <f aca="false">(B15-B14)/D14*100</f>
+        <v>-0.43458828467271</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" s="13" t="n">
+        <v>-18.2</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" s="13" t="n">
         <v>0.1</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="D25" s="13" t="n">
         <v>0.8</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>103</v>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2229,12 +2682,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2242,25 +2695,25 @@
         <v>35</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2268,25 +2721,25 @@
         <v>38</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>100</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="F5" s="13" t="n">
         <v>16630</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2294,35 +2747,35 @@
         <v>41</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>100</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="F6" s="13" t="n">
         <v>15483.733</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>